<commit_message>
Checkpoint before assistant change: Add ability to print receipts for customer purchases
Add a new feature that allows users to print receipts for their transactions.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -452,7 +452,7 @@
         <v>Latest Apple iPhone with advanced camera system</v>
       </c>
       <c r="D2">
-        <v>89999</v>
+        <v>99999</v>
       </c>
       <c r="E2">
         <v>75000</v>
@@ -461,7 +461,7 @@
         <v>Electronics</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -472,11 +472,11 @@
       <c r="J2" t="str">
         <v>APPLE-IP14PRO-128</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2">
         <v>45292</v>
       </c>
       <c r="L2" s="1">
-        <v>45306</v>
+        <v>45903.53644927083</v>
       </c>
     </row>
     <row r="3">
@@ -510,10 +510,10 @@
       <c r="J3" t="str">
         <v>SAMSUNG-GW5-44MM</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3">
         <v>45293</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3">
         <v>45301</v>
       </c>
     </row>
@@ -548,10 +548,10 @@
       <c r="J4" t="str">
         <v>APPLE-MBA-M2-256</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4">
         <v>45294</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4">
         <v>45303</v>
       </c>
     </row>
@@ -586,10 +586,10 @@
       <c r="J5" t="str">
         <v>APPLE-APP-2ND-GEN</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5">
         <v>45295</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5">
         <v>45299</v>
       </c>
     </row>
@@ -624,10 +624,10 @@
       <c r="J6" t="str">
         <v>DELL-XPS13-I7-512</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6">
         <v>45296</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6">
         <v>45305</v>
       </c>
     </row>
@@ -640,7 +640,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -708,7 +708,7 @@
       <c r="I2" t="str">
         <v>Card</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2">
         <v>45306</v>
       </c>
       <c r="K2" t="str">
@@ -746,7 +746,7 @@
       <c r="I3" t="str">
         <v>UPI</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3">
         <v>45307</v>
       </c>
       <c r="K3" t="str">
@@ -784,7 +784,7 @@
       <c r="I4" t="str">
         <v>Card</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <v>45308</v>
       </c>
       <c r="K4" t="str">
@@ -822,7 +822,7 @@
       <c r="I5" t="str">
         <v>Cash</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <v>45309</v>
       </c>
       <c r="K5" t="str">
@@ -832,9 +832,47 @@
         <v>Bulk purchase for team</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>84b542ce-e1a7-4d92-90db-f730d963b3e6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>prod-001</v>
+      </c>
+      <c r="C6" t="str">
+        <v>iPhone 14 Pro</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>99999</v>
+      </c>
+      <c r="F6" t="str">
+        <v>99999</v>
+      </c>
+      <c r="G6" t="str">
+        <v>24999</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Zeeshan</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="J6">
+        <v>45903.53644912037</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -891,7 +929,7 @@
       <c r="F2" t="str">
         <v>Property Management Co.</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>45292</v>
       </c>
       <c r="H2" t="str">
@@ -920,7 +958,7 @@
       <c r="F3" t="str">
         <v>State Electricity Board</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>45296</v>
       </c>
       <c r="H3" t="str">
@@ -949,7 +987,7 @@
       <c r="F4" t="str">
         <v>Facebook Ads</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>45301</v>
       </c>
       <c r="H4" t="str">
@@ -978,7 +1016,7 @@
       <c r="F5" t="str">
         <v>Tech Distributors Ltd.</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>45303</v>
       </c>
       <c r="H5" t="str">
@@ -997,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1044,7 +1082,7 @@
       <c r="F2">
         <v>50</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>45292</v>
       </c>
       <c r="H2" t="str">
@@ -1070,7 +1108,7 @@
       <c r="F3">
         <v>150</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>45292</v>
       </c>
       <c r="H3" t="str">
@@ -1096,16 +1134,42 @@
       <c r="F4">
         <v>600</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>45292</v>
       </c>
       <c r="H4" t="str">
         <v>Active</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>f58f98b7-8249-4761-ac89-b155fe221eb4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2025-09</v>
+      </c>
+      <c r="D5" t="str">
+        <v>10000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>1000</v>
+      </c>
+      <c r="F5">
+        <v>50</v>
+      </c>
+      <c r="G5">
+        <v>45903.535934444444</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint before assistant change: Adjust dashboard layout to prevent content overflow
Update the layout of dashboard components to ensure all content is displayed correctly without overflowing.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -67,9 +67,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -461,7 +460,7 @@
         <v>Electronics</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -475,8 +474,8 @@
       <c r="K2">
         <v>45292</v>
       </c>
-      <c r="L2" s="1">
-        <v>45903.53644927083</v>
+      <c r="L2" t="str">
+        <v>2025-09-03T13:19:39.402Z</v>
       </c>
     </row>
     <row r="3">
@@ -640,7 +639,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -870,9 +869,47 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>39962c9b-8c04-46b9-92ce-fd6a599059c6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>prod-001</v>
+      </c>
+      <c r="C7" t="str">
+        <v>iPhone 14 Pro</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>99999</v>
+      </c>
+      <c r="F7" t="str">
+        <v>99999</v>
+      </c>
+      <c r="G7" t="str">
+        <v>24999</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Zeeshan</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2025-09-03T13:19:39.384Z</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Perform comprehensive cleanup and fix critical Excel import errors
Fixes XLSX import issues in excel-storage.ts by switching to a default import, updates package.json with a new description, and adds LICENSE and README.md files.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 03766aec-11e8-441f-8360-56f12f8d401c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 7cafe6db-f597-40f0-9b2a-a60ccc2fe118
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/fb8e1910-b61f-4ff2-aa01-dfb7adb7be52/03766aec-11e8-441f-8360-56f12f8d401c/CAoFtXv
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -916,7 +916,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1063,16 +1063,42 @@
         <v>Monthly inventory purchase</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>56db455e-58cf-4e50-9f05-e57fe5fbf90d</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Monthly rent</v>
+      </c>
+      <c r="D6" t="str">
+        <v>5000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Landlord</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-05-09T10:06:50.778Z</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1204,9 +1230,35 @@
         <v>Active</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>196eb5bb-a157-42e3-a6a5-3240675be634</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="D6" t="str">
+        <v>100000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>20000</v>
+      </c>
+      <c r="F6">
+        <v>50</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-05-09T10:06:50.853Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add a settings page for managing account and application data
Implement a new settings page with features for changing user passwords, viewing storage statistics, and resetting all application data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 03766aec-11e8-441f-8360-56f12f8d401c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 857c2ad7-4dda-4d66-aa6b-368379433b77
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/fb8e1910-b61f-4ff2-aa01-dfb7adb7be52/03766aec-11e8-441f-8360-56f12f8d401c/6mS1KKQ
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -460,7 +460,7 @@
         <v>Electronics</v>
       </c>
       <c r="G2">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -475,7 +475,7 @@
         <v>45292</v>
       </c>
       <c r="L2" t="str">
-        <v>2025-09-03T13:19:39.402Z</v>
+        <v>2026-05-09T10:10:06.304Z</v>
       </c>
     </row>
     <row r="3">
@@ -498,7 +498,7 @@
         <v>Electronics</v>
       </c>
       <c r="G3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>3</v>
@@ -512,8 +512,8 @@
       <c r="K3">
         <v>45293</v>
       </c>
-      <c r="L3">
-        <v>45301</v>
+      <c r="L3" t="str">
+        <v>2026-05-09T10:11:57.236Z</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +639,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -907,9 +907,85 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1fbf5eed-138e-4108-bdfb-fb60928468b0</v>
+      </c>
+      <c r="B8" t="str">
+        <v>prod-001</v>
+      </c>
+      <c r="C8" t="str">
+        <v>iPhone 14 Pro</v>
+      </c>
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8" t="str">
+        <v>99999</v>
+      </c>
+      <c r="F8" t="str">
+        <v>1299987</v>
+      </c>
+      <c r="G8" t="str">
+        <v>324987</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2026-05-09T10:10:06.283Z</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>9430e9a2-ff3d-4a79-9ed8-8023ab794e26</v>
+      </c>
+      <c r="B9" t="str">
+        <v>prod-002</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Samsung Galaxy Watch 5</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="str">
+        <v>25999</v>
+      </c>
+      <c r="F9" t="str">
+        <v>207992</v>
+      </c>
+      <c r="G9" t="str">
+        <v>47992</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="J9" t="str">
+        <v>2026-05-09T10:11:57.228Z</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove Replit references and add developer social links to settings
Removes Replit script from index.html, removes Replit devDependencies from package.json, syncs package-lock.json, and adds social links to the settings page.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: cdbd3f54-fad5-4082-9744-620eb99e58cb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: dfbc6489-46e5-43fb-9cbe-a56d8e88d77b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/ad721540-aea0-4632-ae78-ffc766d134d2/cdbd3f54-fad5-4082-9744-620eb99e58cb/c2w7Xd6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -400,313 +400,138 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
         <v>name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>description</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>price</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>cost_price</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>category</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>stock</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>min_stock</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>supplier</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>sku</v>
-      </c>
-      <c r="J1" t="str">
-        <v>id</v>
       </c>
       <c r="K1" t="str">
         <v>created_date</v>
       </c>
       <c r="L1" t="str">
         <v>last_updated</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Amul Butter (500g)</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2">
-        <v>500</v>
-      </c>
-      <c r="D2">
-        <v>100</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Food</v>
-      </c>
-      <c r="F2">
-        <v>18</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v>07291cea-a90f-4352-b915-1121e63dcb59</v>
-      </c>
-      <c r="K2" t="str">
-        <v>2025-09-23T12:50:58.115Z</v>
-      </c>
-      <c r="L2" t="str">
-        <v>2025-09-23T13:05:26.195Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
         <v>product_id</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
+        <v>product_name</v>
+      </c>
+      <c r="D1" t="str">
         <v>quantity</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>unit_price</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
+        <v>total_amount</v>
+      </c>
+      <c r="G1" t="str">
+        <v>profit</v>
+      </c>
+      <c r="H1" t="str">
         <v>customer_name</v>
       </c>
-      <c r="E1" t="str">
+      <c r="I1" t="str">
         <v>payment_method</v>
       </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
+        <v>sale_date</v>
+      </c>
+      <c r="K1" t="str">
         <v>cashier</v>
       </c>
-      <c r="G1" t="str">
+      <c r="L1" t="str">
         <v>notes</v>
-      </c>
-      <c r="H1" t="str">
-        <v>id</v>
-      </c>
-      <c r="I1" t="str">
-        <v>product_name</v>
-      </c>
-      <c r="J1" t="str">
-        <v>total_amount</v>
-      </c>
-      <c r="K1" t="str">
-        <v>profit</v>
-      </c>
-      <c r="L1" t="str">
-        <v>sale_date</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>07291cea-a90f-4352-b915-1121e63dcb59</v>
-      </c>
-      <c r="B2">
-        <v>71</v>
-      </c>
-      <c r="C2" t="str">
-        <v>500</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>9cbf4f85-2a79-4a90-8951-8c7ed4927e8d</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Amul Butter (500g)</v>
-      </c>
-      <c r="J2" t="str">
-        <v>35500</v>
-      </c>
-      <c r="K2" t="str">
-        <v>28400</v>
-      </c>
-      <c r="L2" t="str">
-        <v>2025-09-23T12:51:14.506Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>07291cea-a90f-4352-b915-1121e63dcb59</v>
-      </c>
-      <c r="B3">
-        <v>10</v>
-      </c>
-      <c r="C3" t="str">
-        <v>500</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>e66c2199-14fc-46af-b2ee-ed7812584635</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Amul Butter (500g)</v>
-      </c>
-      <c r="J3" t="str">
-        <v>5000</v>
-      </c>
-      <c r="K3" t="str">
-        <v>4000</v>
-      </c>
-      <c r="L3" t="str">
-        <v>2025-09-23T13:02:08.595Z</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>07291cea-a90f-4352-b915-1121e63dcb59</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="str">
-        <v>500</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
-        <v>15ca83ea-a74c-421a-911c-b93c602bde13</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Amul Butter (500g)</v>
-      </c>
-      <c r="J4" t="str">
-        <v>500</v>
-      </c>
-      <c r="K4" t="str">
-        <v>400</v>
-      </c>
-      <c r="L4" t="str">
-        <v>2025-09-23T13:05:26.171Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
         <v>category</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>description</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>amount</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>payment_method</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>vendor</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>expense_date</v>
+      </c>
+      <c r="H1" t="str">
+        <v>receipt_number</v>
+      </c>
+      <c r="I1" t="str">
         <v>notes</v>
-      </c>
-      <c r="G1" t="str">
-        <v>id</v>
-      </c>
-      <c r="H1" t="str">
-        <v>expense_date</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Utilities</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Random</v>
-      </c>
-      <c r="C2" t="str">
-        <v>5000</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Cash</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>0f1d1996-63c0-461d-b044-35309c9cda10</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2025-09-23T12:51:31.350Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update branding and fix receipt printing for desktop and web applications
Removes Replit-specific configurations and code, updates branding in reports and sales pages, and refactors receipt printing to use a consistent window.open method for both web and Electron environments.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: cdbd3f54-fad5-4082-9744-620eb99e58cb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a47b2d21-8f48-43c2-a0a1-c1e8de757a45
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/ad721540-aea0-4632-ae78-ffc766d134d2/cdbd3f54-fad5-4082-9744-620eb99e58cb/c2w7Xd6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/data/shop_data.xlsx
+++ b/data/shop_data.xlsx
@@ -400,98 +400,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>price</v>
+      </c>
+      <c r="D1" t="str">
+        <v>cost_price</v>
+      </c>
+      <c r="E1" t="str">
+        <v>category</v>
+      </c>
+      <c r="F1" t="str">
+        <v>stock</v>
+      </c>
+      <c r="G1" t="str">
+        <v>min_stock</v>
+      </c>
+      <c r="H1" t="str">
+        <v>supplier</v>
+      </c>
+      <c r="I1" t="str">
+        <v>sku</v>
+      </c>
+      <c r="J1" t="str">
         <v>id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>description</v>
-      </c>
-      <c r="D1" t="str">
-        <v>price</v>
-      </c>
-      <c r="E1" t="str">
-        <v>cost_price</v>
-      </c>
-      <c r="F1" t="str">
-        <v>category</v>
-      </c>
-      <c r="G1" t="str">
-        <v>stock</v>
-      </c>
-      <c r="H1" t="str">
-        <v>min_stock</v>
-      </c>
-      <c r="I1" t="str">
-        <v>supplier</v>
-      </c>
-      <c r="J1" t="str">
-        <v>sku</v>
       </c>
       <c r="K1" t="str">
         <v>created_date</v>
       </c>
       <c r="L1" t="str">
         <v>last_updated</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>test</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>100</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Clothing</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v>64f3077a-9c69-43e7-95d8-7538fc1106b1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-05-11T11:29:17.841Z</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-05-11T11:33:35.806Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>product_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>quantity</v>
+      </c>
+      <c r="C1" t="str">
+        <v>unit_price</v>
+      </c>
+      <c r="D1" t="str">
+        <v>customer_name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>payment_method</v>
+      </c>
+      <c r="F1" t="str">
+        <v>cashier</v>
+      </c>
+      <c r="G1" t="str">
+        <v>notes</v>
+      </c>
+      <c r="H1" t="str">
         <v>id</v>
       </c>
-      <c r="B1" t="str">
-        <v>product_id</v>
-      </c>
-      <c r="C1" t="str">
+      <c r="I1" t="str">
         <v>product_name</v>
       </c>
-      <c r="D1" t="str">
-        <v>quantity</v>
-      </c>
-      <c r="E1" t="str">
-        <v>unit_price</v>
-      </c>
-      <c r="F1" t="str">
+      <c r="J1" t="str">
         <v>total_amount</v>
       </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
         <v>profit</v>
       </c>
-      <c r="H1" t="str">
-        <v>customer_name</v>
-      </c>
-      <c r="I1" t="str">
-        <v>payment_method</v>
-      </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>sale_date</v>
       </c>
-      <c r="K1" t="str">
-        <v>cashier</v>
-      </c>
-      <c r="L1" t="str">
-        <v>notes</v>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>64f3077a-9c69-43e7-95d8-7538fc1106b1</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2" t="str">
+        <v>100</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>52e3eeb9-e110-41d2-8616-2eca9bb554fe</v>
+      </c>
+      <c r="I2" t="str">
+        <v>test</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1000</v>
+      </c>
+      <c r="K2" t="str">
+        <v>1000</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-05-11T11:29:22.636Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>